<commit_message>
Sync planning SharePoint : S41
</commit_message>
<xml_diff>
--- a/Plannings 2026 S41.xlsx
+++ b/Plannings 2026 S41.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37694237-19EA-44DF-ACA0-E2985A841EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{37694237-19EA-44DF-ACA0-E2985A841EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67222E19-38C5-4D1B-8A2C-A6B62757C2D3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="120">
   <si>
     <t>Planning des salariés du 05/10/2026 au 11/10/2026</t>
   </si>
@@ -372,9 +372,6 @@
     <t>17:30/22:30</t>
   </si>
   <si>
-    <t>INVENTAIRE // C. PADEL // EVENT SAFRAN PU</t>
-  </si>
-  <si>
     <t>C. PADEL // EDF</t>
   </si>
   <si>
@@ -382,6 +379,9 @@
   </si>
   <si>
     <t>C. PADEL // EDF // LEAGUES</t>
+  </si>
+  <si>
+    <t>C. PADEL // EVENT GTM</t>
   </si>
 </sst>
 </file>
@@ -5406,24 +5406,26 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="36" t="s">
-        <v>119</v>
-      </c>
-      <c r="D3" s="36" t="s">
+      <c r="F3" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="E3" s="36" t="s">
+      <c r="G3" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="F3" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="G3" s="36" t="s">
+      <c r="H3" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="36"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="36" t="s">
@@ -7500,13 +7502,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24D7A2B-9FD9-411E-9456-3A78290D458E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D416C393-5E79-4870-A27A-DCA7B0769528}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFCF5860-6BE1-4684-838A-E84D137BACE4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3D62615-20CC-41D7-9549-DFC38910738C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{880A5CE2-4B9F-4A75-A43E-CA6BA6DAC4DB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B057C25-B0AE-4E3E-88D5-B45C14832292}"/>
 </file>
</xml_diff>